<commit_message>
updated the report 	modified:   main/Multi-Asset Risk Dashboard & Portfolio.docx 	modified:   output/BLO_risk_dashboard.xlsx 	modified:   risk_dashboard/BLO_risk_dashboard.py
</commit_message>
<xml_diff>
--- a/output/BLO_risk_dashboard.xlsx
+++ b/output/BLO_risk_dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/daa8df5e598afa50/KF/projects/Mutli asset risk dashboard portfolio optimization/multi-asset-risk-dashboard-portfolio/output/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="12" documentId="11_D0DA490B8F8326A26DC696AACAB7AB1FB73EA782" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2AC2453-23B1-43A7-AEFC-4180366F16DC}"/>
+  <xr:revisionPtr revIDLastSave="29" documentId="11_D0DA490B8F8326A26DC696AACAB7AB1FB73EA782" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1398459C-6DD7-4A36-B216-47E2ECC56645}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="13" activeTab="15" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" firstSheet="18" activeTab="18" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Summary Metrics" sheetId="1" r:id="rId1"/>
@@ -36,12 +36,25 @@
     <sheet name="Final Risk Contribution Chart" sheetId="21" r:id="rId21"/>
     <sheet name="Rolling Beta and Alpha" sheetId="22" r:id="rId22"/>
   </sheets>
-  <calcPr calcId="124519"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="193" uniqueCount="151">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="151">
   <si>
     <t>Metric</t>
   </si>
@@ -3018,6 +3031,10 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
@@ -3427,7 +3444,7 @@
         <v>14</v>
       </c>
       <c r="B16" s="2">
-        <v>-9.5179129705903573</v>
+        <v>-9.5179129705903601E-2</v>
       </c>
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.35">
@@ -3522,6 +3539,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
   <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -5384,7 +5404,7 @@
   <dimension ref="A1:Y67"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.35">
@@ -12488,6 +12508,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:C55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
@@ -14974,10 +14997,15 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:D55"/>
+  <dimension ref="A1:E55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.81640625" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="21.81640625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>28</v>
       </c>
@@ -14985,13 +15013,16 @@
         <v>39</v>
       </c>
       <c r="C1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D1" t="s">
         <v>40</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4">
         <v>44531</v>
       </c>
@@ -14999,13 +15030,17 @@
         <v>-58.76115852665545</v>
       </c>
       <c r="C2">
+        <f>B2/100</f>
+        <v>-0.58761158526655455</v>
+      </c>
+      <c r="D2">
         <v>55.906134946787553</v>
       </c>
-      <c r="D2">
+      <c r="E2">
         <v>29.020227229963702</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="4">
         <v>44562</v>
       </c>
@@ -15013,13 +15048,17 @@
         <v>-25.535411207226311</v>
       </c>
       <c r="C3">
+        <f t="shared" ref="C3:C55" si="0">B3/100</f>
+        <v>-0.25535411207226311</v>
+      </c>
+      <c r="D3">
         <v>60.701515766562807</v>
       </c>
-      <c r="D3">
+      <c r="E3">
         <v>35.605673122165378</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="4">
         <v>44593</v>
       </c>
@@ -15027,13 +15066,17 @@
         <v>-13.267537913685199</v>
       </c>
       <c r="C4">
+        <f t="shared" si="0"/>
+        <v>-0.13267537913685198</v>
+      </c>
+      <c r="D4">
         <v>59.691104632389823</v>
       </c>
-      <c r="D4">
+      <c r="E4">
         <v>10.100504178246499</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="4">
         <v>44621</v>
       </c>
@@ -15041,13 +15084,17 @@
         <v>-26.386082394246611</v>
       </c>
       <c r="C5">
+        <f t="shared" si="0"/>
+        <v>-0.26386082394246613</v>
+      </c>
+      <c r="D5">
         <v>59.865889900362824</v>
       </c>
-      <c r="D5">
+      <c r="E5">
         <v>29.251272471918551</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="4">
         <v>44652</v>
       </c>
@@ -15055,13 +15102,17 @@
         <v>-9.0564683887952562</v>
       </c>
       <c r="C6">
+        <f t="shared" si="0"/>
+        <v>-9.0564683887952566E-2</v>
+      </c>
+      <c r="D6">
         <v>56.436506436164471</v>
       </c>
-      <c r="D6">
+      <c r="E6">
         <v>44.741002745719101</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="4">
         <v>44682</v>
       </c>
@@ -15069,13 +15120,17 @@
         <v>-6.4128477055492699</v>
       </c>
       <c r="C7">
+        <f t="shared" si="0"/>
+        <v>-6.4128477055492697E-2</v>
+      </c>
+      <c r="D7">
         <v>57.412035199643597</v>
       </c>
-      <c r="D7">
+      <c r="E7">
         <v>44.741002745719101</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="4">
         <v>44713</v>
       </c>
@@ -15083,13 +15138,17 @@
         <v>8.438014954569077</v>
       </c>
       <c r="C8">
+        <f t="shared" si="0"/>
+        <v>8.4380149545690772E-2</v>
+      </c>
+      <c r="D8">
         <v>58.424437283595182</v>
       </c>
-      <c r="D8">
+      <c r="E8">
         <v>52.903497578694306</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A9" s="4">
         <v>44743</v>
       </c>
@@ -15097,13 +15156,17 @@
         <v>-1.7900280260487761E-2</v>
       </c>
       <c r="C9">
+        <f t="shared" si="0"/>
+        <v>-1.790028026048776E-4</v>
+      </c>
+      <c r="D9">
         <v>58.553759314755048</v>
       </c>
-      <c r="D9">
+      <c r="E9">
         <v>52.903497578694306</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="4">
         <v>44774</v>
       </c>
@@ -15111,13 +15174,17 @@
         <v>10.890134674001191</v>
       </c>
       <c r="C10">
+        <f t="shared" si="0"/>
+        <v>0.10890134674001191</v>
+      </c>
+      <c r="D10">
         <v>59.070131146434107</v>
       </c>
-      <c r="D10">
+      <c r="E10">
         <v>55.591521825013679</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A11" s="4">
         <v>44805</v>
       </c>
@@ -15125,13 +15192,17 @@
         <v>12.28976787449254</v>
       </c>
       <c r="C11">
+        <f t="shared" si="0"/>
+        <v>0.1228976787449254</v>
+      </c>
+      <c r="D11">
         <v>59.070131146434107</v>
       </c>
-      <c r="D11">
+      <c r="E11">
         <v>59.746577030609771</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="4">
         <v>44835</v>
       </c>
@@ -15139,13 +15210,17 @@
         <v>46.298653256933747</v>
       </c>
       <c r="C12">
+        <f t="shared" si="0"/>
+        <v>0.46298653256933747</v>
+      </c>
+      <c r="D12">
         <v>99.726908684657175</v>
       </c>
-      <c r="D12">
+      <c r="E12">
         <v>59.746577030609771</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="4">
         <v>44866</v>
       </c>
@@ -15153,13 +15228,17 @@
         <v>41.924842149605119</v>
       </c>
       <c r="C13">
+        <f t="shared" si="0"/>
+        <v>0.41924842149605118</v>
+      </c>
+      <c r="D13">
         <v>96.000823833508576</v>
       </c>
-      <c r="D13">
+      <c r="E13">
         <v>59.746577030609771</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="4">
         <v>44896</v>
       </c>
@@ -15167,13 +15246,17 @@
         <v>44.658787965846543</v>
       </c>
       <c r="C14">
+        <f t="shared" si="0"/>
+        <v>0.44658787965846541</v>
+      </c>
+      <c r="D14">
         <v>96.000823833508576</v>
       </c>
-      <c r="D14">
+      <c r="E14">
         <v>61.555640091028188</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="4">
         <v>44927</v>
       </c>
@@ -15181,13 +15264,17 @@
         <v>25.073803424213761</v>
       </c>
       <c r="C15">
+        <f t="shared" si="0"/>
+        <v>0.25073803424213759</v>
+      </c>
+      <c r="D15">
         <v>89.222330912507843</v>
       </c>
-      <c r="D15">
+      <c r="E15">
         <v>65.662128258879747</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="4">
         <v>44958</v>
       </c>
@@ -15195,13 +15282,17 @@
         <v>20.15502547030756</v>
       </c>
       <c r="C16">
+        <f t="shared" si="0"/>
+        <v>0.20155025470307561</v>
+      </c>
+      <c r="D16">
         <v>93.072479088251214</v>
       </c>
-      <c r="D16">
+      <c r="E16">
         <v>73.539796873843059</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="4">
         <v>44986</v>
       </c>
@@ -15209,13 +15300,17 @@
         <v>12.15065813460442</v>
       </c>
       <c r="C17">
+        <f t="shared" si="0"/>
+        <v>0.1215065813460442</v>
+      </c>
+      <c r="D17">
         <v>87.964707801130047</v>
       </c>
-      <c r="D17">
+      <c r="E17">
         <v>73.539796873843059</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="4">
         <v>45017</v>
       </c>
@@ -15223,13 +15318,17 @@
         <v>-1.6147703878691479</v>
       </c>
       <c r="C18">
+        <f t="shared" si="0"/>
+        <v>-1.614770387869148E-2</v>
+      </c>
+      <c r="D18">
         <v>86.082446985163074</v>
       </c>
-      <c r="D18">
+      <c r="E18">
         <v>79.181268543288127</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="4">
         <v>45047</v>
       </c>
@@ -15237,13 +15336,17 @@
         <v>-18.395841379005631</v>
       </c>
       <c r="C19">
+        <f t="shared" si="0"/>
+        <v>-0.18395841379005631</v>
+      </c>
+      <c r="D19">
         <v>75.976482233310946</v>
       </c>
-      <c r="D19">
+      <c r="E19">
         <v>79.181268543288127</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="4">
         <v>45078</v>
       </c>
@@ -15251,13 +15354,17 @@
         <v>-22.95961388586279</v>
       </c>
       <c r="C20">
+        <f t="shared" si="0"/>
+        <v>-0.2295961388586279</v>
+      </c>
+      <c r="D20">
         <v>77.511700008556801</v>
       </c>
-      <c r="D20">
+      <c r="E20">
         <v>80.073451018988763</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A21" s="4">
         <v>45108</v>
       </c>
@@ -15265,13 +15372,17 @@
         <v>-19.015923342455199</v>
       </c>
       <c r="C21">
+        <f t="shared" si="0"/>
+        <v>-0.19015923342455199</v>
+      </c>
+      <c r="D21">
         <v>78.666491470587658</v>
       </c>
-      <c r="D21">
+      <c r="E21">
         <v>80.073451018988763</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="4">
         <v>45139</v>
       </c>
@@ -15279,13 +15390,17 @@
         <v>-25.08796197659116</v>
       </c>
       <c r="C22">
+        <f t="shared" si="0"/>
+        <v>-0.25087961976591161</v>
+      </c>
+      <c r="D22">
         <v>78.113659900761789</v>
       </c>
-      <c r="D22">
+      <c r="E22">
         <v>84.68251869833351</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="4">
         <v>45170</v>
       </c>
@@ -15293,13 +15408,17 @@
         <v>-26.671652912473661</v>
       </c>
       <c r="C23">
+        <f t="shared" si="0"/>
+        <v>-0.26671652912473659</v>
+      </c>
+      <c r="D23">
         <v>78.113659900761789</v>
       </c>
-      <c r="D23">
+      <c r="E23">
         <v>84.68945542933028</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A24" s="4">
         <v>45200</v>
       </c>
@@ -15307,13 +15426,17 @@
         <v>-48.063592416685061</v>
       </c>
       <c r="C24">
+        <f t="shared" si="0"/>
+        <v>-0.48063592416685064</v>
+      </c>
+      <c r="D24">
         <v>63.973775859674909</v>
       </c>
-      <c r="D24">
+      <c r="E24">
         <v>61.228959460365758</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="4">
         <v>45231</v>
       </c>
@@ -15321,13 +15444,17 @@
         <v>-48.939456235103442</v>
       </c>
       <c r="C25">
+        <f t="shared" si="0"/>
+        <v>-0.4893945623510344</v>
+      </c>
+      <c r="D25">
         <v>61.808966106710969</v>
       </c>
-      <c r="D25">
+      <c r="E25">
         <v>61.228959460365758</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="4">
         <v>45261</v>
       </c>
@@ -15335,13 +15462,17 @@
         <v>-60.580858243392228</v>
       </c>
       <c r="C26">
+        <f t="shared" si="0"/>
+        <v>-0.60580858243392233</v>
+      </c>
+      <c r="D26">
         <v>62.380593611693058</v>
       </c>
-      <c r="D26">
+      <c r="E26">
         <v>53.723995387342093</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A27" s="4">
         <v>45292</v>
       </c>
@@ -15349,13 +15480,17 @@
         <v>-63.09902433036526</v>
       </c>
       <c r="C27">
+        <f t="shared" si="0"/>
+        <v>-0.63099024330365261</v>
+      </c>
+      <c r="D27">
         <v>58.297673244461969</v>
       </c>
-      <c r="D27">
+      <c r="E27">
         <v>53.723995387342093</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A28" s="4">
         <v>45323</v>
       </c>
@@ -15363,13 +15498,17 @@
         <v>-79.8015316298183</v>
       </c>
       <c r="C28">
+        <f t="shared" si="0"/>
+        <v>-0.79801531629818301</v>
+      </c>
+      <c r="D28">
         <v>53.74681446751152</v>
       </c>
-      <c r="D28">
+      <c r="E28">
         <v>53.723995387342093</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A29" s="4">
         <v>45352</v>
       </c>
@@ -15377,13 +15516,17 @@
         <v>-68.369390864996433</v>
       </c>
       <c r="C29">
+        <f t="shared" si="0"/>
+        <v>-0.68369390864996438</v>
+      </c>
+      <c r="D29">
         <v>56.899541600074279</v>
       </c>
-      <c r="D29">
+      <c r="E29">
         <v>53.723995387342093</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A30" s="4">
         <v>45383</v>
       </c>
@@ -15391,13 +15534,17 @@
         <v>-55.186157542221103</v>
       </c>
       <c r="C30">
+        <f t="shared" si="0"/>
+        <v>-0.55186157542221104</v>
+      </c>
+      <c r="D30">
         <v>58.321494797736072</v>
       </c>
-      <c r="D30">
+      <c r="E30">
         <v>46.514134359686317</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A31" s="4">
         <v>45413</v>
       </c>
@@ -15405,13 +15552,17 @@
         <v>-52.767512871468391</v>
       </c>
       <c r="C31">
+        <f t="shared" si="0"/>
+        <v>-0.52767512871468392</v>
+      </c>
+      <c r="D31">
         <v>63.888438699985429</v>
       </c>
-      <c r="D31">
+      <c r="E31">
         <v>46.514134359686317</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A32" s="4">
         <v>45444</v>
       </c>
@@ -15419,13 +15570,17 @@
         <v>-64.019276610271106</v>
       </c>
       <c r="C32">
+        <f t="shared" si="0"/>
+        <v>-0.64019276610271103</v>
+      </c>
+      <c r="D32">
         <v>58.483739337698239</v>
       </c>
-      <c r="D32">
+      <c r="E32">
         <v>46.514134359686317</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A33" s="4">
         <v>45474</v>
       </c>
@@ -15433,13 +15588,17 @@
         <v>-27.058325191463471</v>
       </c>
       <c r="C33">
+        <f t="shared" si="0"/>
+        <v>-0.27058325191463473</v>
+      </c>
+      <c r="D33">
         <v>59.368710383179888</v>
       </c>
-      <c r="D33">
+      <c r="E33">
         <v>5.2288282937396717</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A34" s="4">
         <v>45505</v>
       </c>
@@ -15447,13 +15606,17 @@
         <v>-23.797777695019061</v>
       </c>
       <c r="C34">
+        <f t="shared" si="0"/>
+        <v>-0.23797777695019062</v>
+      </c>
+      <c r="D34">
         <v>61.936708508101233</v>
       </c>
-      <c r="D34">
+      <c r="E34">
         <v>5.2288282937396717</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A35" s="4">
         <v>45536</v>
       </c>
@@ -15461,13 +15624,17 @@
         <v>-25.595634986531699</v>
       </c>
       <c r="C35">
+        <f t="shared" si="0"/>
+        <v>-0.25595634986531701</v>
+      </c>
+      <c r="D35">
         <v>62.14172736404349</v>
       </c>
-      <c r="D35">
+      <c r="E35">
         <v>-79.928793757677553</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A36" s="4">
         <v>45566</v>
       </c>
@@ -15475,13 +15642,17 @@
         <v>-38.469054746563891</v>
       </c>
       <c r="C36">
+        <f t="shared" si="0"/>
+        <v>-0.38469054746563891</v>
+      </c>
+      <c r="D36">
         <v>59.903784417750728</v>
       </c>
-      <c r="D36">
+      <c r="E36">
         <v>-39.400756939787193</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A37" s="4">
         <v>45597</v>
       </c>
@@ -15489,13 +15660,17 @@
         <v>-33.921570631132113</v>
       </c>
       <c r="C37">
+        <f t="shared" si="0"/>
+        <v>-0.33921570631132114</v>
+      </c>
+      <c r="D37">
         <v>58.911199934797303</v>
       </c>
-      <c r="D37">
+      <c r="E37">
         <v>-39.400756939787193</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A38" s="4">
         <v>45627</v>
       </c>
@@ -15503,13 +15678,17 @@
         <v>-39.995182316160381</v>
       </c>
       <c r="C38">
+        <f t="shared" si="0"/>
+        <v>-0.39995182316160383</v>
+      </c>
+      <c r="D38">
         <v>50.55144128335273</v>
       </c>
-      <c r="D38">
+      <c r="E38">
         <v>-39.400756939787193</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A39" s="4">
         <v>45658</v>
       </c>
@@ -15517,13 +15696,17 @@
         <v>-27.9079367344278</v>
       </c>
       <c r="C39">
+        <f t="shared" si="0"/>
+        <v>-0.27907936734427802</v>
+      </c>
+      <c r="D39">
         <v>52.416761620926209</v>
       </c>
-      <c r="D39">
+      <c r="E39">
         <v>0.93355035873024117</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A40" s="4">
         <v>45689</v>
       </c>
@@ -15531,13 +15714,17 @@
         <v>-12.94081668607722</v>
       </c>
       <c r="C40">
+        <f t="shared" si="0"/>
+        <v>-0.12940816686077219</v>
+      </c>
+      <c r="D40">
         <v>49.057524346629243</v>
       </c>
-      <c r="D40">
+      <c r="E40">
         <v>-0.35449662824740569</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A41" s="4">
         <v>45717</v>
       </c>
@@ -15545,13 +15732,17 @@
         <v>-4.8518539791405511</v>
       </c>
       <c r="C41">
+        <f t="shared" si="0"/>
+        <v>-4.851853979140551E-2</v>
+      </c>
+      <c r="D41">
         <v>40.808507985589337</v>
       </c>
-      <c r="D41">
+      <c r="E41">
         <v>23.97932791841281</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A42" s="4">
         <v>45748</v>
       </c>
@@ -15559,13 +15750,17 @@
         <v>-13.33458154742355</v>
       </c>
       <c r="C42">
+        <f t="shared" si="0"/>
+        <v>-0.13334581547423549</v>
+      </c>
+      <c r="D42">
         <v>43.798160645257568</v>
       </c>
-      <c r="D42">
+      <c r="E42">
         <v>21.59836026748804</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A43" s="4">
         <v>45778</v>
       </c>
@@ -15573,13 +15768,17 @@
         <v>-18.720976112816889</v>
       </c>
       <c r="C43">
+        <f t="shared" si="0"/>
+        <v>-0.18720976112816889</v>
+      </c>
+      <c r="D43">
         <v>43.05219117262714</v>
       </c>
-      <c r="D43">
+      <c r="E43">
         <v>21.59836026748804</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A44" s="4">
         <v>45809</v>
       </c>
@@ -15587,13 +15786,17 @@
         <v>-20.942220944263291</v>
       </c>
       <c r="C44">
+        <f t="shared" si="0"/>
+        <v>-0.2094222094426329</v>
+      </c>
+      <c r="D44">
         <v>43.172632338177621</v>
       </c>
-      <c r="D44">
+      <c r="E44">
         <v>21.59836026748804</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A45" s="4">
         <v>45839</v>
       </c>
@@ -15601,13 +15804,17 @@
         <v>-60.423455198366348</v>
       </c>
       <c r="C45">
+        <f t="shared" si="0"/>
+        <v>-0.60423455198366349</v>
+      </c>
+      <c r="D45">
         <v>40.400282405106097</v>
       </c>
-      <c r="D45">
+      <c r="E45">
         <v>59.113127907006373</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A46" s="4">
         <v>45870</v>
       </c>
@@ -15615,13 +15822,17 @@
         <v>-45.975227423594632</v>
       </c>
       <c r="C46">
+        <f t="shared" si="0"/>
+        <v>-0.45975227423594633</v>
+      </c>
+      <c r="D46">
         <v>36.329694785384731</v>
       </c>
-      <c r="D46">
+      <c r="E46">
         <v>38.1287064733324</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A47" s="4">
         <v>45901</v>
       </c>
@@ -15629,13 +15840,17 @@
         <v>-40.146765051598457</v>
       </c>
       <c r="C47">
+        <f t="shared" si="0"/>
+        <v>-0.4014676505159846</v>
+      </c>
+      <c r="D47">
         <v>43.833040283935169</v>
       </c>
-      <c r="D47">
+      <c r="E47">
         <v>38.1287064733324</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A48" s="4">
         <v>45931</v>
       </c>
@@ -15643,13 +15858,17 @@
         <v>-42.3478462882263</v>
       </c>
       <c r="C48">
+        <f t="shared" si="0"/>
+        <v>-0.42347846288226298</v>
+      </c>
+      <c r="D48">
         <v>48.170429742750812</v>
       </c>
-      <c r="D48">
+      <c r="E48">
         <v>38.1287064733324</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A49" s="4">
         <v>45962</v>
       </c>
@@ -15657,13 +15876,17 @@
         <v>-37.487290916453773</v>
       </c>
       <c r="C49">
+        <f t="shared" si="0"/>
+        <v>-0.37487290916453775</v>
+      </c>
+      <c r="D49">
         <v>50.123383304200608</v>
       </c>
-      <c r="D49">
+      <c r="E49">
         <v>55.755588470264733</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A50" s="4">
         <v>45992</v>
       </c>
@@ -15671,13 +15894,17 @@
         <v>-18.94491418513433</v>
       </c>
       <c r="C50">
+        <f t="shared" si="0"/>
+        <v>-0.18944914185134329</v>
+      </c>
+      <c r="D50">
         <v>58.258878485609813</v>
       </c>
-      <c r="D50">
+      <c r="E50">
         <v>41.384761878345152</v>
       </c>
     </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A51" s="4">
         <v>46023</v>
       </c>
@@ -15685,13 +15912,17 @@
         <v>4.4929706539922636</v>
       </c>
       <c r="C51">
+        <f t="shared" si="0"/>
+        <v>4.4929706539922634E-2</v>
+      </c>
+      <c r="D51">
         <v>58.258878485609813</v>
       </c>
-      <c r="D51">
+      <c r="E51">
         <v>-25.074559329973479</v>
       </c>
     </row>
-    <row r="52" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A52" s="4">
         <v>46054</v>
       </c>
@@ -15699,13 +15930,17 @@
         <v>7.4626237505683806</v>
       </c>
       <c r="C52">
+        <f t="shared" si="0"/>
+        <v>7.4626237505683812E-2</v>
+      </c>
+      <c r="D52">
         <v>58.258878485609813</v>
       </c>
-      <c r="D52">
+      <c r="E52">
         <v>-18.43312473761112</v>
       </c>
     </row>
-    <row r="53" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A53" s="4">
         <v>46082</v>
       </c>
@@ -15713,13 +15948,17 @@
         <v>8.5588679950914272E-3</v>
       </c>
       <c r="C53">
+        <f t="shared" si="0"/>
+        <v>8.5588679950914266E-5</v>
+      </c>
+      <c r="D53">
         <v>58.258878485609813</v>
       </c>
-      <c r="D53">
+      <c r="E53">
         <v>-34.680092173256</v>
       </c>
     </row>
-    <row r="54" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A54" s="4">
         <v>46113</v>
       </c>
@@ -15727,13 +15966,17 @@
         <v>-12.93394607433984</v>
       </c>
       <c r="C54">
+        <f t="shared" si="0"/>
+        <v>-0.12933946074339839</v>
+      </c>
+      <c r="D54">
         <v>50.784427272381357</v>
       </c>
-      <c r="D54">
+      <c r="E54">
         <v>-34.680092173256</v>
       </c>
     </row>
-    <row r="55" spans="1:4" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A55" s="4">
         <v>46143</v>
       </c>
@@ -15741,9 +15984,13 @@
         <v>-9.5179129705903573</v>
       </c>
       <c r="C55">
+        <f t="shared" si="0"/>
+        <v>-9.5179129705903573E-2</v>
+      </c>
+      <c r="D55">
         <v>49.589308832178787</v>
       </c>
-      <c r="D55">
+      <c r="E55">
         <v>-34.680092173256</v>
       </c>
     </row>
@@ -15756,6 +16003,9 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:C66"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="17.81640625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.35">
       <c r="A1" t="s">

</xml_diff>